<commit_message>
Populate Korean template with sample content
Co-authored-by: TWBSY <nnmnsalmon@gmail.com>
</commit_message>
<xml_diff>
--- a/gacha_design_template_ko.xlsx
+++ b/gacha_design_template_ko.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -475,15 +475,219 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>EVT_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>환율 급등</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>환율이 9 이하일 때</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>90초</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>환전 보너스 +5%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>환율</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>환율 화살표+반짝</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>EVT_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>시장 폭락</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>시세계수 0.8 미만</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>판매가 -15%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>붉은 그래프</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>EVT_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>수상한 상인 방문</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>상인</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>상인 해금 후 5분 주기</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>특수 매입/판매 열림</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>상인</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>어두운 조명</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>EVT_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>첫 SSR 획득</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>스토리</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SSR 최초 획득</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>즉시</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>축하 보상 코인 +50,000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>황금 연출</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>EVT_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>투자 대박 찬스</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>시스템</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>원화 1,000만 이상</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>120초</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>고위험 투자 상품 임시 오픈</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>투자</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>폭죽</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -496,7 +700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -537,13 +741,169 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>환율</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>10 코인=1원</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>±5%</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>N 시세</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>90초</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>±5~10%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R 시세</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>90초</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>±10~20%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SR 시세</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>90초</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>±10~25%</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2.5</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SSR 시세</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>90초</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>±5~15%</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>0.5</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -556,7 +916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -592,12 +952,88 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>END_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>기본 엔딩</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>원화 5,000만 달성</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>엔딩 컷신</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>도전과제 오픈</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>END_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>투자 대박 엔딩</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>투자 수익률 누적 +200%</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>특수 컷신</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>고액 목표 해금</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>END_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>블랙마켓 엔딩</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>암시장 거래 10회</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>비밀 엔딩</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>도감 확장</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -610,7 +1046,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -651,13 +1087,169 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>UI_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>메인(코인 탭)</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>가챠/현황 표시</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>기본 진입</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>가챠 버튼</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>코인/원화/진행률</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>UI_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>가챠 결과</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>결과 표시/판매</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>가챠 후</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>바로 판매</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>아이템 정보</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>UI_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>인벤토리</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>보관/판매/정렬</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>기본 해금</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>판매</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>아이템 리스트</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>UI_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>업그레이드</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>구매/효과 확인</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>기본 해금</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>구매</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>업그레이드 카드</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>UI_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>원화 탭</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>환전/투자/룰렛</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>열쇠 구매 후</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>환전</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>환율/원화</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -670,7 +1262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -721,15 +1313,227 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SYS_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>1연차 무료 가챠</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>코어 루프 진입</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>아이템 1개</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>기본 해금</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>메인</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SYS_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10연차 가챠+스킵</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>플레이 템포 개선</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>아이템 10개</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>기본 해금</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>스킵 시 신규 아이템 연출</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>SYS_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>인벤토리 정렬/필터</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>판매 효율 개선</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>정렬/필터 적용</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>기본 해금</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>중간</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>인벤토리</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>SYS_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>코인→원화 환전</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>원화 콘텐츠 진입</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>코인</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>원화</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>열쇠 구매 후</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>원화탭</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>환율 변동 적용</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SYS_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>룰렛 베팅</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>리스크/보상 선택지</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>원화</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>배당 결과</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>원화 탭 해금 후</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>중간</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>원화탭</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -742,7 +1546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -808,18 +1612,560 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>N_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>고장난 키링</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>320</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>260</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>잡화</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>특별한 효과 없음</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>N_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>중고 스티커</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>220</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>380</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>잡화</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>수집용</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>R_001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>한정판 굿즈</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1000</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1800</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1400</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>컬렉션</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>시세에 민감</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>R_002</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>레어 사인 카드</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>1200</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1600</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>컬렉션</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>콜렉터가 선호</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>SR_001</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>블루칩 투자권</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>10000</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>8000</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>투자</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>판매 시 고수익</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>SR_002</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>프리미엄 티켓</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>6000</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>12000</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>9000</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>이벤트</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>특수 상인 선호</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>SSR_001</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>황금 주식권</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>SSR</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>30000</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>80000</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>60000</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>투자;희귀</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>개별 시세 적용</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>SSR_002</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>블랙 카드</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>SSR</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>90000</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>65000</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VIP</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>상인이 고가 매입</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SP_001</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>VIP 초대장</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>키</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>키</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>이벤트 분기 진입</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>이벤트</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>SP_002</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>내부 정보 서류</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Special</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>키</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>키</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>투자 찬스 이벤트</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>특수 상인</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>아니오</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -832,7 +2178,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -878,14 +2224,80 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>SET_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>증권가 세트</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>블루칩 투자권;황금 주식권;증권 리포트</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>투자 수익률 +5%p</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>세트 3종 보유</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SR</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>낮음</t>
+        </is>
+      </c>
       <c r="H2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>SET_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VIP 룸 세트</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>블랙 카드;VIP 초대장;프리미엄 티켓</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>상인 매입가 +10%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>세트 3종 보유</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>SSR</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>낮음</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -898,7 +2310,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -939,13 +2351,70 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>KEY_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>VIP 초대장</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>VIP 엔딩 분기</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>이벤트/가챠</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>중간</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>KEY_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>내부 정보 서류</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>투자 대박 이벤트</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>예</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>특수 상인</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>중간</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -958,7 +2427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:N3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1034,20 +2503,124 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>BN_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>기본 무료 배너</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>일반 풀</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>65%</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>22%</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.5%</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>기본/10연차</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>10연차 스킵 가능</t>
+        </is>
+      </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>BN_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>세트 픽업 배너</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>세트 아이템 비중↑</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>60%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>24%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>12%</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>3%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>1%</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>SR 1개 보장</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>특수 연출</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>스킵 시 신규 연출</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1060,7 +2633,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1111,15 +2684,219 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>UP_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>판매가 보너스 I</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>수익</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>기본 해금</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>10,000~83,000</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>레벨당 +20%</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>모든 아이템 판매가 증가</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>UP_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>판매가 보너스 II</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>수익</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>원화 500만</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>100,000~490,000</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>레벨당 +25%</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>후반 전체 판매가 강화</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>UP_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>운세 상승</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>가챠</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>판매가 보너스 I 3레벨</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>50,000~150,000</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>고등급 확률 상승</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>조금 더 높은 등급이 나옵니다</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>UP_004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>시장 안전망</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>시장</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>원화 200만</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>30,000~150,000</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>최소 시세계수 +0.05</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>폭락 방지</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>UP_005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>수상한 상인 소개</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>특수</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>판매가 보너스 I 2레벨</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>50,000</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>상인 등장</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>특수 상인 해금</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1132,7 +2909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1188,16 +2965,148 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>MCH_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>코인 중개인</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5분</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>일반;잡화</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>일반 아이템</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>없음</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>MCH_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>컬렉터</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5분</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>세트;컬렉션</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>세트 아이템</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>0.9</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>세트 이벤트</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>MCH_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>암시장 상인</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>7분</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>60초</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>희귀;키</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>특수 아이템</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>0.7</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>비밀 이벤트</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1210,7 +3119,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1266,16 +3175,148 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr"/>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>INV_001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>예금</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>5분</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>+5%</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>+5% 고정</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>낮음</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>500만</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>제한 없음</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>원화 탭 해금</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>INV_002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>채권형</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>5분</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>+7~8%</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>-5%~+20%</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>중간</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>500만</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>현재 원화의 50%</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>원화 탭 해금</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>INV_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>주식형</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>5분</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>+25%</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>-50%~+100%</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>500만</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>현재 원화의 30%</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>원화 탭 해금</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>